<commit_message>
Pipeline: scrape legacy + contrôle croisé (12Z)
</commit_message>
<xml_diff>
--- a/legacy/Forecast-19102026-12Z.xlsx
+++ b/legacy/Forecast-19102026-12Z.xlsx
@@ -635,7 +635,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 20/10/2026 01:04</t>
+          <t>Généré le : 21/10/2026 00:36</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1775,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 20/10/2026 01:04</t>
+          <t>Généré le : 21/10/2026 00:36</t>
         </is>
       </c>
     </row>
@@ -26263,7 +26263,7 @@
         <v>1.9</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H21" s="19" t="n">
         <v>-1.3</v>
@@ -26557,7 +26557,7 @@
         <v>-1.5</v>
       </c>
       <c r="AG23" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AH23" s="19" t="n">
         <v>-0.2</v>
@@ -26593,7 +26593,7 @@
         <v>-1.2</v>
       </c>
       <c r="I24" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="J24" s="19" t="n">
         <v>-1.4</v>
@@ -28093,7 +28093,7 @@
         <v>1.4</v>
       </c>
       <c r="E38" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F38" s="18" t="n">
         <v>0.8</v>
@@ -28126,7 +28126,7 @@
         <v>-0.8</v>
       </c>
       <c r="P38" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q38" s="18" t="n">
         <v>0.1</v>
@@ -28525,7 +28525,7 @@
         <v>-1.1</v>
       </c>
       <c r="E42" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F42" s="19" t="n">
         <v>-1.5</v>
@@ -28570,7 +28570,7 @@
         <v>-1.8</v>
       </c>
       <c r="T42" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="U42" s="19" t="n">
         <v>-0.9</v>
@@ -28660,7 +28660,7 @@
         <v>-0.9</v>
       </c>
       <c r="N43" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O43" s="21" t="n">
         <v>-3.8</v>
@@ -28798,7 +28798,7 @@
         <v>0.4</v>
       </c>
       <c r="X44" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Y44" s="19" t="n">
         <v>-0.7</v>
@@ -28954,7 +28954,7 @@
         <v>0.8</v>
       </c>
       <c r="D46" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E46" s="18" t="n">
         <v>1.6</v>
@@ -29014,7 +29014,7 @@
         <v>2.1</v>
       </c>
       <c r="X46" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Y46" s="18" t="n">
         <v>0.1</v>
@@ -29080,7 +29080,7 @@
         <v>3.9</v>
       </c>
       <c r="J47" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>0.1</v>
@@ -29203,7 +29203,7 @@
         <v>8.199999999999999</v>
       </c>
       <c r="O48" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="P48" s="13" t="n">
         <v>7.6</v>
@@ -30421,7 +30421,7 @@
         <v>7.8</v>
       </c>
       <c r="Y59" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z59" s="13" t="n">
         <v>6.9</v>
@@ -30448,7 +30448,7 @@
         <v>-0.8</v>
       </c>
       <c r="AH59" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -31792,7 +31792,7 @@
         <v>0.1</v>
       </c>
       <c r="N72" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O72" s="13" t="n">
         <v>6.6</v>
@@ -31804,7 +31804,7 @@
         <v>5.7</v>
       </c>
       <c r="R72" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="S72" s="12" t="n">
         <v>4.1</v>
@@ -32905,7 +32905,7 @@
         <v>6.5</v>
       </c>
       <c r="Y82" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z82" s="13" t="n">
         <v>6.4</v>
@@ -33163,7 +33163,7 @@
         </is>
       </c>
       <c r="C85" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="D85" s="17" t="n">
         <v>3.9</v>

</xml_diff>